<commit_message>
memperbaiki fitur import dan double email
</commit_message>
<xml_diff>
--- a/public/referensi/import-user management-role-user.xlsx
+++ b/public/referensi/import-user management-role-user.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADVAN\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\aset-mgmt\public\referensi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4CDA03B-0DF9-48D4-9C88-7C39677D7CCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96414E7E-3C80-4D69-96AB-934E3B21B877}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
     <author>Poltekpar Lombok</author>
   </authors>
   <commentList>
-    <comment ref="A119" authorId="0" shapeId="0" xr:uid="{0016C350-9341-4086-BF21-F4415E93F02E}">
+    <comment ref="A118" authorId="0" shapeId="0" xr:uid="{0016C350-9341-4086-BF21-F4415E93F02E}">
       <text>
         <r>
           <rPr>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="406">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="406">
   <si>
     <t>fullname</t>
   </si>
@@ -1070,9 +1070,6 @@
     <t>PassSapa112</t>
   </si>
   <si>
-    <t>Yusup Apriyanto, S.Pd</t>
-  </si>
-  <si>
     <t>Adam Rahmadi Akbar, A.Md.Par., S.Tr.Par</t>
   </si>
   <si>
@@ -1160,18 +1157,12 @@
     <t>haris@ppl.ac.id</t>
   </si>
   <si>
-    <t>pati@ppl.ac.id</t>
-  </si>
-  <si>
     <t>yulia@ppl.ac.id</t>
   </si>
   <si>
     <t>tsabiatun@ppl.ac.id</t>
   </si>
   <si>
-    <t>PassSapa113</t>
-  </si>
-  <si>
     <t>PassSapa114</t>
   </si>
   <si>
@@ -1272,6 +1263,15 @@
   </si>
   <si>
     <t>PassSapa135</t>
+  </si>
+  <si>
+    <t>putu@ppl.ac.id</t>
+  </si>
+  <si>
+    <t>sahroni@ppl.ac.id</t>
+  </si>
+  <si>
+    <t>Ertonpati@ppl.ac.id</t>
   </si>
 </sst>
 </file>
@@ -1493,7 +1493,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1502,16 +1502,16 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1520,35 +1520,29 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1569,7 +1563,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -1580,11 +1573,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1914,12 +1903,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D136"/>
+  <dimension ref="A1:D135"/>
   <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="76" customWidth="1"/>
     <col min="2" max="2" width="22.3984375" customWidth="1"/>
-    <col min="3" max="3" width="37" style="32" customWidth="1"/>
+    <col min="3" max="3" width="37" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1930,7 +1919,7 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="27" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -1941,19 +1930,19 @@
       <c r="A2" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="20" t="str">
+      <c r="B2" s="18" t="str">
         <f>LEFT(C2, FIND("@", C2) - 1)</f>
         <v>komangmahawira</v>
       </c>
-      <c r="C2" s="28" t="s">
+      <c r="C2" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="19" t="s">
         <v>226</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="9" t="s">
         <v>5</v>
       </c>
       <c r="B3" s="2" t="str">
@@ -1963,12 +1952,12 @@
       <c r="C3" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="D3" s="21" t="s">
+      <c r="D3" s="19" t="s">
         <v>227</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="11" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="2" t="str">
@@ -1978,12 +1967,12 @@
       <c r="C4" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="D4" s="21" t="s">
+      <c r="D4" s="19" t="s">
         <v>228</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="14" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="11" t="s">
         <v>119</v>
       </c>
       <c r="B5" s="2" t="str">
@@ -1993,12 +1982,12 @@
       <c r="C5" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="D5" s="21" t="s">
+      <c r="D5" s="19" t="s">
         <v>229</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="9" t="s">
         <v>7</v>
       </c>
       <c r="B6" s="2" t="str">
@@ -2008,7 +1997,7 @@
       <c r="C6" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="D6" s="21" t="s">
+      <c r="D6" s="19" t="s">
         <v>230</v>
       </c>
     </row>
@@ -2023,12 +2012,12 @@
       <c r="C7" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="D7" s="21" t="s">
+      <c r="D7" s="19" t="s">
         <v>231</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="9" t="s">
         <v>9</v>
       </c>
       <c r="B8" s="2" t="str">
@@ -2038,12 +2027,12 @@
       <c r="C8" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="D8" s="21" t="s">
+      <c r="D8" s="19" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="9" t="s">
         <v>10</v>
       </c>
       <c r="B9" s="2" t="str">
@@ -2053,12 +2042,12 @@
       <c r="C9" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="D9" s="21" t="s">
+      <c r="D9" s="19" t="s">
         <v>233</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="9" t="s">
         <v>11</v>
       </c>
       <c r="B10" s="2" t="str">
@@ -2068,12 +2057,12 @@
       <c r="C10" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="D10" s="21" t="s">
+      <c r="D10" s="19" t="s">
         <v>234</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="9" t="s">
         <v>12</v>
       </c>
       <c r="B11" s="2" t="str">
@@ -2083,12 +2072,12 @@
       <c r="C11" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="D11" s="21" t="s">
+      <c r="D11" s="19" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="9" t="s">
         <v>13</v>
       </c>
       <c r="B12" s="2" t="str">
@@ -2098,12 +2087,12 @@
       <c r="C12" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D12" s="21" t="s">
+      <c r="D12" s="19" t="s">
         <v>236</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="9" t="s">
         <v>14</v>
       </c>
       <c r="B13" s="2" t="str">
@@ -2113,12 +2102,12 @@
       <c r="C13" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="D13" s="21" t="s">
+      <c r="D13" s="19" t="s">
         <v>237</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="9" t="s">
         <v>15</v>
       </c>
       <c r="B14" s="2" t="str">
@@ -2128,12 +2117,12 @@
       <c r="C14" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="D14" s="21" t="s">
+      <c r="D14" s="19" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="9" t="s">
         <v>16</v>
       </c>
       <c r="B15" s="2" t="str">
@@ -2143,12 +2132,12 @@
       <c r="C15" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="D15" s="21" t="s">
+      <c r="D15" s="19" t="s">
         <v>239</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="9" t="s">
         <v>17</v>
       </c>
       <c r="B16" s="2" t="str">
@@ -2158,12 +2147,12 @@
       <c r="C16" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="D16" s="21" t="s">
+      <c r="D16" s="19" t="s">
         <v>240</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="12" t="s">
         <v>18</v>
       </c>
       <c r="B17" s="2" t="str">
@@ -2173,12 +2162,12 @@
       <c r="C17" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="D17" s="21" t="s">
+      <c r="D17" s="19" t="s">
         <v>241</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="9" t="s">
         <v>19</v>
       </c>
       <c r="B18" s="2" t="str">
@@ -2188,12 +2177,12 @@
       <c r="C18" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="D18" s="21" t="s">
+      <c r="D18" s="19" t="s">
         <v>242</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A19" s="13" t="s">
+      <c r="A19" s="12" t="s">
         <v>20</v>
       </c>
       <c r="B19" s="2" t="str">
@@ -2203,12 +2192,12 @@
       <c r="C19" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="D19" s="21" t="s">
+      <c r="D19" s="19" t="s">
         <v>243</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="9" t="s">
         <v>21</v>
       </c>
       <c r="B20" s="2" t="str">
@@ -2218,12 +2207,12 @@
       <c r="C20" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="D20" s="21" t="s">
+      <c r="D20" s="19" t="s">
         <v>244</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A21" s="11" t="s">
+      <c r="A21" s="9" t="s">
         <v>22</v>
       </c>
       <c r="B21" s="2" t="str">
@@ -2233,12 +2222,12 @@
       <c r="C21" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="D21" s="21" t="s">
+      <c r="D21" s="19" t="s">
         <v>245</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A22" s="11" t="s">
+      <c r="A22" s="9" t="s">
         <v>23</v>
       </c>
       <c r="B22" s="2" t="str">
@@ -2248,12 +2237,12 @@
       <c r="C22" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D22" s="21" t="s">
+      <c r="D22" s="19" t="s">
         <v>246</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="14" t="s">
+      <c r="A23" s="13" t="s">
         <v>24</v>
       </c>
       <c r="B23" s="2" t="str">
@@ -2263,12 +2252,12 @@
       <c r="C23" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="D23" s="21" t="s">
+      <c r="D23" s="19" t="s">
         <v>247</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A24" s="15" t="s">
+      <c r="A24" s="14" t="s">
         <v>25</v>
       </c>
       <c r="B24" s="2" t="str">
@@ -2278,12 +2267,12 @@
       <c r="C24" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D24" s="21" t="s">
+      <c r="D24" s="19" t="s">
         <v>248</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A25" s="11" t="s">
+      <c r="A25" s="9" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="2" t="str">
@@ -2293,12 +2282,12 @@
       <c r="C25" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="D25" s="21" t="s">
+      <c r="D25" s="19" t="s">
         <v>249</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A26" s="11" t="s">
+      <c r="A26" s="9" t="s">
         <v>27</v>
       </c>
       <c r="B26" s="2" t="str">
@@ -2308,12 +2297,12 @@
       <c r="C26" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="D26" s="21" t="s">
+      <c r="D26" s="19" t="s">
         <v>250</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A27" s="15" t="s">
+      <c r="A27" s="14" t="s">
         <v>28</v>
       </c>
       <c r="B27" s="2" t="str">
@@ -2323,12 +2312,12 @@
       <c r="C27" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="D27" s="21" t="s">
+      <c r="D27" s="19" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A28" s="11" t="s">
+      <c r="A28" s="9" t="s">
         <v>29</v>
       </c>
       <c r="B28" s="2" t="str">
@@ -2338,12 +2327,12 @@
       <c r="C28" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="D28" s="21" t="s">
+      <c r="D28" s="19" t="s">
         <v>252</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A29" s="15" t="s">
+      <c r="A29" s="14" t="s">
         <v>30</v>
       </c>
       <c r="B29" s="2" t="str">
@@ -2353,12 +2342,12 @@
       <c r="C29" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="D29" s="21" t="s">
+      <c r="D29" s="19" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A30" s="12" t="s">
+      <c r="A30" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B30" s="2" t="str">
@@ -2368,12 +2357,12 @@
       <c r="C30" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D30" s="21" t="s">
+      <c r="D30" s="19" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A31" s="11" t="s">
+      <c r="A31" s="9" t="s">
         <v>32</v>
       </c>
       <c r="B31" s="2" t="str">
@@ -2383,27 +2372,27 @@
       <c r="C31" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="D31" s="21" t="s">
+      <c r="D31" s="19" t="s">
         <v>255</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A32" s="11" t="s">
+      <c r="A32" s="9" t="s">
         <v>33</v>
       </c>
       <c r="B32" s="2" t="str">
         <f t="shared" si="0"/>
-        <v>ari</v>
+        <v>putu</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="D32" s="21" t="s">
+        <v>403</v>
+      </c>
+      <c r="D32" s="19" t="s">
         <v>256</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A33" s="11" t="s">
+      <c r="A33" s="9" t="s">
         <v>34</v>
       </c>
       <c r="B33" s="2" t="str">
@@ -2413,12 +2402,12 @@
       <c r="C33" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="D33" s="21" t="s">
+      <c r="D33" s="19" t="s">
         <v>257</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A34" s="16" t="s">
+      <c r="A34" s="15" t="s">
         <v>35</v>
       </c>
       <c r="B34" s="2" t="str">
@@ -2428,12 +2417,12 @@
       <c r="C34" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="D34" s="21" t="s">
+      <c r="D34" s="19" t="s">
         <v>258</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A35" s="11" t="s">
+      <c r="A35" s="9" t="s">
         <v>36</v>
       </c>
       <c r="B35" s="2" t="str">
@@ -2443,12 +2432,12 @@
       <c r="C35" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="D35" s="21" t="s">
+      <c r="D35" s="19" t="s">
         <v>259</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A36" s="11" t="s">
+      <c r="A36" s="9" t="s">
         <v>37</v>
       </c>
       <c r="B36" s="2" t="str">
@@ -2458,12 +2447,12 @@
       <c r="C36" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="D36" s="21" t="s">
+      <c r="D36" s="19" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A37" s="17" t="s">
+      <c r="A37" s="16" t="s">
         <v>38</v>
       </c>
       <c r="B37" s="2" t="str">
@@ -2473,12 +2462,12 @@
       <c r="C37" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="D37" s="21" t="s">
+      <c r="D37" s="19" t="s">
         <v>261</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A38" s="18" t="s">
+      <c r="A38" s="17" t="s">
         <v>39</v>
       </c>
       <c r="B38" s="2" t="str">
@@ -2488,12 +2477,12 @@
       <c r="C38" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="D38" s="21" t="s">
+      <c r="D38" s="19" t="s">
         <v>262</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A39" s="15" t="s">
+      <c r="A39" s="14" t="s">
         <v>40</v>
       </c>
       <c r="B39" s="2" t="str">
@@ -2503,12 +2492,12 @@
       <c r="C39" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="D39" s="21" t="s">
+      <c r="D39" s="19" t="s">
         <v>263</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A40" s="15" t="s">
+      <c r="A40" s="14" t="s">
         <v>41</v>
       </c>
       <c r="B40" s="2" t="str">
@@ -2518,12 +2507,12 @@
       <c r="C40" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="D40" s="21" t="s">
+      <c r="D40" s="19" t="s">
         <v>264</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A41" s="16" t="s">
+      <c r="A41" s="15" t="s">
         <v>81</v>
       </c>
       <c r="B41" s="2" t="str">
@@ -2533,12 +2522,12 @@
       <c r="C41" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="D41" s="21" t="s">
+      <c r="D41" s="19" t="s">
         <v>265</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A42" s="16" t="s">
+      <c r="A42" s="15" t="s">
         <v>82</v>
       </c>
       <c r="B42" s="2" t="str">
@@ -2548,12 +2537,12 @@
       <c r="C42" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="D42" s="21" t="s">
+      <c r="D42" s="19" t="s">
         <v>266</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A43" s="16" t="s">
+      <c r="A43" s="15" t="s">
         <v>83</v>
       </c>
       <c r="B43" s="2" t="str">
@@ -2563,12 +2552,12 @@
       <c r="C43" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="D43" s="21" t="s">
+      <c r="D43" s="19" t="s">
         <v>267</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="19" t="s">
+      <c r="A44" s="3" t="s">
         <v>84</v>
       </c>
       <c r="B44" s="2" t="str">
@@ -2578,12 +2567,12 @@
       <c r="C44" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="D44" s="21" t="s">
+      <c r="D44" s="19" t="s">
         <v>268</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A45" s="16" t="s">
+      <c r="A45" s="15" t="s">
         <v>85</v>
       </c>
       <c r="B45" s="2" t="str">
@@ -2593,12 +2582,12 @@
       <c r="C45" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="D45" s="21" t="s">
+      <c r="D45" s="19" t="s">
         <v>269</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A46" s="16" t="s">
+      <c r="A46" s="15" t="s">
         <v>86</v>
       </c>
       <c r="B46" s="2" t="str">
@@ -2608,12 +2597,12 @@
       <c r="C46" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="D46" s="21" t="s">
+      <c r="D46" s="19" t="s">
         <v>270</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A47" s="16" t="s">
+      <c r="A47" s="15" t="s">
         <v>87</v>
       </c>
       <c r="B47" s="2" t="str">
@@ -2623,12 +2612,12 @@
       <c r="C47" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="D47" s="21" t="s">
+      <c r="D47" s="19" t="s">
         <v>271</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A48" s="16" t="s">
+      <c r="A48" s="15" t="s">
         <v>88</v>
       </c>
       <c r="B48" s="2" t="str">
@@ -2638,12 +2627,12 @@
       <c r="C48" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="D48" s="21" t="s">
+      <c r="D48" s="19" t="s">
         <v>272</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A49" s="16" t="s">
+      <c r="A49" s="15" t="s">
         <v>89</v>
       </c>
       <c r="B49" s="2" t="str">
@@ -2653,12 +2642,12 @@
       <c r="C49" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="D49" s="21" t="s">
+      <c r="D49" s="19" t="s">
         <v>273</v>
       </c>
     </row>
     <row r="50" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A50" s="16" t="s">
+      <c r="A50" s="15" t="s">
         <v>90</v>
       </c>
       <c r="B50" s="2" t="str">
@@ -2668,117 +2657,117 @@
       <c r="C50" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="D50" s="21" t="s">
+      <c r="D50" s="19" t="s">
         <v>274</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A51" s="16" t="s">
+      <c r="A51" s="15" t="s">
         <v>120</v>
       </c>
       <c r="B51" s="2" t="str">
         <f t="shared" si="0"/>
         <v>mala</v>
       </c>
-      <c r="C51" s="29" t="s">
+      <c r="C51" s="26" t="s">
         <v>125</v>
       </c>
-      <c r="D51" s="21" t="s">
+      <c r="D51" s="19" t="s">
         <v>275</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A52" s="16" t="s">
+      <c r="A52" s="15" t="s">
         <v>121</v>
       </c>
       <c r="B52" s="2" t="str">
         <f t="shared" si="0"/>
         <v>ari</v>
       </c>
-      <c r="C52" s="29" t="s">
+      <c r="C52" s="26" t="s">
         <v>72</v>
       </c>
-      <c r="D52" s="21" t="s">
+      <c r="D52" s="19" t="s">
         <v>276</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A53" s="16" t="s">
+      <c r="A53" s="15" t="s">
         <v>122</v>
       </c>
       <c r="B53" s="2" t="str">
         <f t="shared" si="0"/>
         <v>hikmatul</v>
       </c>
-      <c r="C53" s="29" t="s">
+      <c r="C53" s="26" t="s">
         <v>124</v>
       </c>
-      <c r="D53" s="21" t="s">
+      <c r="D53" s="19" t="s">
         <v>277</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A54" s="16" t="s">
+      <c r="A54" s="15" t="s">
         <v>101</v>
       </c>
       <c r="B54" s="2" t="str">
         <f t="shared" si="0"/>
         <v>marnishidayah</v>
       </c>
-      <c r="C54" s="30" t="s">
+      <c r="C54" s="27" t="s">
         <v>110</v>
       </c>
-      <c r="D54" s="21" t="s">
+      <c r="D54" s="19" t="s">
         <v>278</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A55" s="16" t="s">
+      <c r="A55" s="15" t="s">
         <v>102</v>
       </c>
       <c r="B55" s="2" t="str">
         <f t="shared" si="0"/>
         <v>rizhkidwiputra</v>
       </c>
-      <c r="C55" s="16" t="s">
+      <c r="C55" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="D55" s="21" t="s">
+      <c r="D55" s="19" t="s">
         <v>279</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A56" s="16" t="s">
+      <c r="A56" s="15" t="s">
         <v>103</v>
       </c>
       <c r="B56" s="2" t="str">
         <f t="shared" si="0"/>
         <v>ayu5made</v>
       </c>
-      <c r="C56" s="30" t="s">
+      <c r="C56" s="27" t="s">
         <v>112</v>
       </c>
-      <c r="D56" s="21" t="s">
+      <c r="D56" s="19" t="s">
         <v>280</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A57" s="16" t="s">
+      <c r="A57" s="15" t="s">
         <v>104</v>
       </c>
       <c r="B57" s="2" t="str">
         <f t="shared" si="0"/>
         <v>seftiasuwari</v>
       </c>
-      <c r="C57" s="16" t="s">
+      <c r="C57" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="D57" s="21" t="s">
+      <c r="D57" s="19" t="s">
         <v>281</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A58" s="16" t="s">
+      <c r="A58" s="15" t="s">
         <v>105</v>
       </c>
       <c r="B58" s="2" t="str">
@@ -2788,12 +2777,12 @@
       <c r="C58" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="D58" s="21" t="s">
+      <c r="D58" s="19" t="s">
         <v>282</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A59" s="16" t="s">
+      <c r="A59" s="15" t="s">
         <v>106</v>
       </c>
       <c r="B59" s="2" t="str">
@@ -2803,12 +2792,12 @@
       <c r="C59" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="D59" s="21" t="s">
+      <c r="D59" s="19" t="s">
         <v>283</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A60" s="16" t="s">
+      <c r="A60" s="15" t="s">
         <v>107</v>
       </c>
       <c r="B60" s="2" t="str">
@@ -2818,12 +2807,12 @@
       <c r="C60" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="D60" s="21" t="s">
+      <c r="D60" s="19" t="s">
         <v>284</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A61" s="16" t="s">
+      <c r="A61" s="15" t="s">
         <v>108</v>
       </c>
       <c r="B61" s="2" t="str">
@@ -2833,12 +2822,12 @@
       <c r="C61" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="D61" s="21" t="s">
+      <c r="D61" s="19" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A62" s="16" t="s">
+      <c r="A62" s="15" t="s">
         <v>109</v>
       </c>
       <c r="B62" s="2" t="str">
@@ -2848,22 +2837,22 @@
       <c r="C62" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="D62" s="21" t="s">
+      <c r="D62" s="19" t="s">
         <v>286</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A63" s="16" t="s">
+      <c r="A63" s="15" t="s">
         <v>123</v>
       </c>
       <c r="B63" s="2" t="str">
         <f t="shared" si="0"/>
-        <v>fahman.toriki007</v>
+        <v>sahroni</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D63" s="21" t="s">
+        <v>404</v>
+      </c>
+      <c r="D63" s="19" t="s">
         <v>287</v>
       </c>
     </row>
@@ -2878,7 +2867,7 @@
       <c r="C64" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="D64" s="21" t="s">
+      <c r="D64" s="19" t="s">
         <v>288</v>
       </c>
     </row>
@@ -2893,7 +2882,7 @@
       <c r="C65" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="D65" s="21" t="s">
+      <c r="D65" s="19" t="s">
         <v>289</v>
       </c>
     </row>
@@ -2908,7 +2897,7 @@
       <c r="C66" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="D66" s="21" t="s">
+      <c r="D66" s="19" t="s">
         <v>290</v>
       </c>
     </row>
@@ -2917,13 +2906,13 @@
         <v>129</v>
       </c>
       <c r="B67" s="2" t="str">
-        <f t="shared" ref="B67:B131" si="1">LEFT(C67, FIND("@", C67) - 1)</f>
+        <f t="shared" ref="B67:B130" si="1">LEFT(C67, FIND("@", C67) - 1)</f>
         <v>sultan.hali</v>
       </c>
       <c r="C67" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="D67" s="21" t="s">
+      <c r="D67" s="19" t="s">
         <v>291</v>
       </c>
     </row>
@@ -2938,7 +2927,7 @@
       <c r="C68" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="D68" s="21" t="s">
+      <c r="D68" s="19" t="s">
         <v>292</v>
       </c>
     </row>
@@ -2950,10 +2939,10 @@
         <f t="shared" si="1"/>
         <v>ilham</v>
       </c>
-      <c r="C69" s="11" t="s">
+      <c r="C69" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="D69" s="21" t="s">
+      <c r="D69" s="19" t="s">
         <v>293</v>
       </c>
     </row>
@@ -2965,10 +2954,10 @@
         <f t="shared" si="1"/>
         <v>hendra</v>
       </c>
-      <c r="C70" s="31" t="s">
+      <c r="C70" s="28" t="s">
         <v>164</v>
       </c>
-      <c r="D70" s="21" t="s">
+      <c r="D70" s="19" t="s">
         <v>294</v>
       </c>
     </row>
@@ -2983,7 +2972,7 @@
       <c r="C71" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="D71" s="21" t="s">
+      <c r="D71" s="19" t="s">
         <v>295</v>
       </c>
     </row>
@@ -2995,10 +2984,10 @@
         <f t="shared" si="1"/>
         <v>m.taupik</v>
       </c>
-      <c r="C72" s="11" t="s">
+      <c r="C72" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="D72" s="21" t="s">
+      <c r="D72" s="19" t="s">
         <v>296</v>
       </c>
     </row>
@@ -3010,10 +2999,10 @@
         <f t="shared" si="1"/>
         <v>akbar</v>
       </c>
-      <c r="C73" s="11" t="s">
+      <c r="C73" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="D73" s="21" t="s">
+      <c r="D73" s="19" t="s">
         <v>297</v>
       </c>
     </row>
@@ -3025,10 +3014,10 @@
         <f t="shared" si="1"/>
         <v>rezakurniawanabka</v>
       </c>
-      <c r="C74" s="11" t="s">
+      <c r="C74" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="D74" s="21" t="s">
+      <c r="D74" s="19" t="s">
         <v>298</v>
       </c>
     </row>
@@ -3040,10 +3029,10 @@
         <f t="shared" si="1"/>
         <v>yus</v>
       </c>
-      <c r="C75" s="11" t="s">
+      <c r="C75" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="D75" s="21" t="s">
+      <c r="D75" s="19" t="s">
         <v>299</v>
       </c>
     </row>
@@ -3058,7 +3047,7 @@
       <c r="C76" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="D76" s="21" t="s">
+      <c r="D76" s="19" t="s">
         <v>300</v>
       </c>
     </row>
@@ -3070,10 +3059,10 @@
         <f t="shared" si="1"/>
         <v>nusyawayaw26</v>
       </c>
-      <c r="C77" s="11" t="s">
+      <c r="C77" s="9" t="s">
         <v>170</v>
       </c>
-      <c r="D77" s="21" t="s">
+      <c r="D77" s="19" t="s">
         <v>301</v>
       </c>
     </row>
@@ -3088,12 +3077,12 @@
       <c r="C78" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="D78" s="21" t="s">
+      <c r="D78" s="19" t="s">
         <v>302</v>
       </c>
     </row>
     <row r="79" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A79" s="22" t="s">
+      <c r="A79" s="20" t="s">
         <v>141</v>
       </c>
       <c r="B79" s="2" t="str">
@@ -3103,12 +3092,12 @@
       <c r="C79" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="D79" s="21" t="s">
+      <c r="D79" s="19" t="s">
         <v>303</v>
       </c>
     </row>
     <row r="80" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A80" s="22" t="s">
+      <c r="A80" s="20" t="s">
         <v>142</v>
       </c>
       <c r="B80" s="2" t="str">
@@ -3118,12 +3107,12 @@
       <c r="C80" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="D80" s="21" t="s">
+      <c r="D80" s="19" t="s">
         <v>304</v>
       </c>
     </row>
     <row r="81" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A81" s="22" t="s">
+      <c r="A81" s="20" t="s">
         <v>143</v>
       </c>
       <c r="B81" s="2" t="str">
@@ -3133,12 +3122,12 @@
       <c r="C81" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="D81" s="21" t="s">
+      <c r="D81" s="19" t="s">
         <v>305</v>
       </c>
     </row>
     <row r="82" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A82" s="23" t="s">
+      <c r="A82" s="21" t="s">
         <v>144</v>
       </c>
       <c r="B82" s="2" t="str">
@@ -3148,12 +3137,12 @@
       <c r="C82" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="D82" s="21" t="s">
+      <c r="D82" s="19" t="s">
         <v>306</v>
       </c>
     </row>
     <row r="83" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A83" s="22" t="s">
+      <c r="A83" s="20" t="s">
         <v>145</v>
       </c>
       <c r="B83" s="2" t="str">
@@ -3163,12 +3152,12 @@
       <c r="C83" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="D83" s="21" t="s">
+      <c r="D83" s="19" t="s">
         <v>307</v>
       </c>
     </row>
     <row r="84" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A84" s="23" t="s">
+      <c r="A84" s="21" t="s">
         <v>146</v>
       </c>
       <c r="B84" s="2" t="str">
@@ -3178,12 +3167,12 @@
       <c r="C84" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="D84" s="21" t="s">
+      <c r="D84" s="19" t="s">
         <v>308</v>
       </c>
     </row>
     <row r="85" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A85" s="23" t="s">
+      <c r="A85" s="21" t="s">
         <v>147</v>
       </c>
       <c r="B85" s="2" t="str">
@@ -3193,12 +3182,12 @@
       <c r="C85" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="D85" s="21" t="s">
+      <c r="D85" s="19" t="s">
         <v>309</v>
       </c>
     </row>
     <row r="86" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A86" s="23" t="s">
+      <c r="A86" s="21" t="s">
         <v>148</v>
       </c>
       <c r="B86" s="2" t="str">
@@ -3208,12 +3197,12 @@
       <c r="C86" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="D86" s="21" t="s">
+      <c r="D86" s="19" t="s">
         <v>310</v>
       </c>
     </row>
     <row r="87" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A87" s="23" t="s">
+      <c r="A87" s="21" t="s">
         <v>149</v>
       </c>
       <c r="B87" s="2" t="str">
@@ -3223,12 +3212,12 @@
       <c r="C87" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="D87" s="21" t="s">
+      <c r="D87" s="19" t="s">
         <v>311</v>
       </c>
     </row>
     <row r="88" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A88" s="22" t="s">
+      <c r="A88" s="20" t="s">
         <v>150</v>
       </c>
       <c r="B88" s="2" t="str">
@@ -3238,7 +3227,7 @@
       <c r="C88" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="D88" s="21" t="s">
+      <c r="D88" s="19" t="s">
         <v>312</v>
       </c>
     </row>
@@ -3253,12 +3242,12 @@
       <c r="C89" s="6" t="s">
         <v>183</v>
       </c>
-      <c r="D89" s="21" t="s">
+      <c r="D89" s="19" t="s">
         <v>313</v>
       </c>
     </row>
     <row r="90" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A90" s="23" t="s">
+      <c r="A90" s="21" t="s">
         <v>152</v>
       </c>
       <c r="B90" s="2" t="str">
@@ -3268,12 +3257,12 @@
       <c r="C90" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="D90" s="21" t="s">
+      <c r="D90" s="19" t="s">
         <v>314</v>
       </c>
     </row>
     <row r="91" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A91" s="22" t="s">
+      <c r="A91" s="20" t="s">
         <v>153</v>
       </c>
       <c r="B91" s="2" t="str">
@@ -3283,12 +3272,12 @@
       <c r="C91" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="D91" s="21" t="s">
+      <c r="D91" s="19" t="s">
         <v>315</v>
       </c>
     </row>
     <row r="92" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A92" s="22" t="s">
+      <c r="A92" s="20" t="s">
         <v>154</v>
       </c>
       <c r="B92" s="2" t="str">
@@ -3298,7 +3287,7 @@
       <c r="C92" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="D92" s="21" t="s">
+      <c r="D92" s="19" t="s">
         <v>316</v>
       </c>
     </row>
@@ -3313,7 +3302,7 @@
       <c r="C93" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="D93" s="21" t="s">
+      <c r="D93" s="19" t="s">
         <v>317</v>
       </c>
     </row>
@@ -3328,7 +3317,7 @@
       <c r="C94" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="D94" s="21" t="s">
+      <c r="D94" s="19" t="s">
         <v>318</v>
       </c>
     </row>
@@ -3343,488 +3332,488 @@
       <c r="C95" s="6" t="s">
         <v>189</v>
       </c>
-      <c r="D95" s="21" t="s">
+      <c r="D95" s="19" t="s">
         <v>319</v>
       </c>
     </row>
     <row r="96" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A96" s="22" t="s">
+      <c r="A96" s="20" t="s">
         <v>190</v>
       </c>
       <c r="B96" s="2" t="str">
         <f t="shared" si="1"/>
         <v>kadek</v>
       </c>
-      <c r="C96" s="29" t="s">
+      <c r="C96" s="26" t="s">
         <v>208</v>
       </c>
-      <c r="D96" s="21" t="s">
+      <c r="D96" s="19" t="s">
         <v>320</v>
       </c>
     </row>
     <row r="97" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A97" s="22" t="s">
+      <c r="A97" s="20" t="s">
         <v>191</v>
       </c>
       <c r="B97" s="2" t="str">
         <f t="shared" si="1"/>
         <v>sopia</v>
       </c>
-      <c r="C97" s="29" t="s">
+      <c r="C97" s="26" t="s">
         <v>209</v>
       </c>
-      <c r="D97" s="21" t="s">
+      <c r="D97" s="19" t="s">
         <v>321</v>
       </c>
     </row>
     <row r="98" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A98" s="22" t="s">
+      <c r="A98" s="20" t="s">
         <v>192</v>
       </c>
       <c r="B98" s="2" t="str">
         <f t="shared" si="1"/>
         <v>diahmustika</v>
       </c>
-      <c r="C98" s="29" t="s">
+      <c r="C98" s="26" t="s">
         <v>212</v>
       </c>
-      <c r="D98" s="21" t="s">
+      <c r="D98" s="19" t="s">
         <v>322</v>
       </c>
     </row>
     <row r="99" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A99" s="23" t="s">
+      <c r="A99" s="21" t="s">
         <v>193</v>
       </c>
       <c r="B99" s="2" t="str">
         <f t="shared" si="1"/>
         <v>desyputri</v>
       </c>
-      <c r="C99" s="29" t="s">
+      <c r="C99" s="26" t="s">
         <v>213</v>
       </c>
-      <c r="D99" s="21" t="s">
+      <c r="D99" s="19" t="s">
         <v>323</v>
       </c>
     </row>
     <row r="100" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A100" s="22" t="s">
+      <c r="A100" s="20" t="s">
         <v>194</v>
       </c>
       <c r="B100" s="2" t="str">
         <f t="shared" si="1"/>
         <v>dora</v>
       </c>
-      <c r="C100" s="29" t="s">
+      <c r="C100" s="26" t="s">
         <v>210</v>
       </c>
-      <c r="D100" s="21" t="s">
+      <c r="D100" s="19" t="s">
         <v>324</v>
       </c>
     </row>
     <row r="101" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A101" s="24" t="s">
+      <c r="A101" s="22" t="s">
         <v>195</v>
       </c>
       <c r="B101" s="2" t="str">
         <f t="shared" si="1"/>
         <v>jaka</v>
       </c>
-      <c r="C101" s="29" t="s">
+      <c r="C101" s="26" t="s">
         <v>214</v>
       </c>
-      <c r="D101" s="21" t="s">
+      <c r="D101" s="19" t="s">
         <v>325</v>
       </c>
     </row>
     <row r="102" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A102" s="23" t="s">
+      <c r="A102" s="21" t="s">
         <v>196</v>
       </c>
       <c r="B102" s="2" t="str">
         <f t="shared" si="1"/>
         <v>didi</v>
       </c>
-      <c r="C102" s="29" t="s">
+      <c r="C102" s="26" t="s">
         <v>211</v>
       </c>
-      <c r="D102" s="21" t="s">
+      <c r="D102" s="19" t="s">
         <v>326</v>
       </c>
     </row>
     <row r="103" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A103" s="24" t="s">
+      <c r="A103" s="22" t="s">
         <v>197</v>
       </c>
       <c r="B103" s="2" t="str">
         <f t="shared" si="1"/>
         <v>yona</v>
       </c>
-      <c r="C103" s="29" t="s">
+      <c r="C103" s="26" t="s">
         <v>215</v>
       </c>
-      <c r="D103" s="21" t="s">
+      <c r="D103" s="19" t="s">
         <v>327</v>
       </c>
     </row>
     <row r="104" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A104" s="24" t="s">
+      <c r="A104" s="22" t="s">
         <v>198</v>
       </c>
       <c r="B104" s="2" t="str">
         <f t="shared" si="1"/>
         <v>astiardi</v>
       </c>
-      <c r="C104" s="29" t="s">
+      <c r="C104" s="26" t="s">
         <v>216</v>
       </c>
-      <c r="D104" s="21" t="s">
+      <c r="D104" s="19" t="s">
         <v>328</v>
       </c>
     </row>
     <row r="105" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A105" s="25" t="s">
+      <c r="A105" s="23" t="s">
         <v>199</v>
       </c>
       <c r="B105" s="2" t="str">
         <f t="shared" si="1"/>
         <v>darsa</v>
       </c>
-      <c r="C105" s="29" t="s">
+      <c r="C105" s="26" t="s">
         <v>217</v>
       </c>
-      <c r="D105" s="21" t="s">
+      <c r="D105" s="19" t="s">
         <v>329</v>
       </c>
     </row>
     <row r="106" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A106" s="26" t="s">
+      <c r="A106" s="24" t="s">
         <v>200</v>
       </c>
       <c r="B106" s="2" t="str">
         <f t="shared" si="1"/>
         <v>hadi</v>
       </c>
-      <c r="C106" s="29" t="s">
+      <c r="C106" s="26" t="s">
         <v>218</v>
       </c>
-      <c r="D106" s="21" t="s">
+      <c r="D106" s="19" t="s">
         <v>330</v>
       </c>
     </row>
     <row r="107" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A107" s="24" t="s">
+      <c r="A107" s="22" t="s">
         <v>201</v>
       </c>
       <c r="B107" s="2" t="str">
         <f t="shared" si="1"/>
         <v>dianAndayani</v>
       </c>
-      <c r="C107" s="29" t="s">
+      <c r="C107" s="26" t="s">
         <v>219</v>
       </c>
-      <c r="D107" s="21" t="s">
+      <c r="D107" s="19" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="108" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A108" s="24" t="s">
+      <c r="A108" s="22" t="s">
         <v>202</v>
       </c>
       <c r="B108" s="2" t="str">
         <f t="shared" si="1"/>
         <v>supardi</v>
       </c>
-      <c r="C108" s="29" t="s">
+      <c r="C108" s="26" t="s">
         <v>220</v>
       </c>
-      <c r="D108" s="21" t="s">
+      <c r="D108" s="19" t="s">
         <v>332</v>
       </c>
     </row>
     <row r="109" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A109" s="25" t="s">
+      <c r="A109" s="23" t="s">
         <v>203</v>
       </c>
       <c r="B109" s="2" t="str">
         <f t="shared" si="1"/>
         <v>surayal</v>
       </c>
-      <c r="C109" s="29" t="s">
+      <c r="C109" s="26" t="s">
         <v>221</v>
       </c>
-      <c r="D109" s="21" t="s">
+      <c r="D109" s="19" t="s">
         <v>333</v>
       </c>
     </row>
     <row r="110" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A110" s="24" t="s">
+      <c r="A110" s="22" t="s">
         <v>204</v>
       </c>
       <c r="B110" s="2" t="str">
         <f t="shared" si="1"/>
         <v>ainul</v>
       </c>
-      <c r="C110" s="29" t="s">
+      <c r="C110" s="26" t="s">
         <v>222</v>
       </c>
-      <c r="D110" s="21" t="s">
+      <c r="D110" s="19" t="s">
         <v>334</v>
       </c>
     </row>
     <row r="111" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A111" s="25" t="s">
+      <c r="A111" s="23" t="s">
         <v>205</v>
       </c>
       <c r="B111" s="2" t="str">
         <f t="shared" si="1"/>
         <v>herlina</v>
       </c>
-      <c r="C111" s="29" t="s">
+      <c r="C111" s="26" t="s">
         <v>223</v>
       </c>
-      <c r="D111" s="21" t="s">
+      <c r="D111" s="19" t="s">
         <v>335</v>
       </c>
     </row>
     <row r="112" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A112" s="24" t="s">
+      <c r="A112" s="22" t="s">
         <v>206</v>
       </c>
       <c r="B112" s="2" t="str">
         <f t="shared" si="1"/>
         <v>lathifah</v>
       </c>
-      <c r="C112" s="29" t="s">
+      <c r="C112" s="26" t="s">
         <v>224</v>
       </c>
-      <c r="D112" s="21" t="s">
+      <c r="D112" s="19" t="s">
         <v>336</v>
       </c>
     </row>
     <row r="113" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A113" s="24" t="s">
+      <c r="A113" s="22" t="s">
         <v>207</v>
       </c>
       <c r="B113" s="2" t="str">
         <f t="shared" si="1"/>
         <v>AhmadZaki</v>
       </c>
-      <c r="C113" s="29" t="s">
+      <c r="C113" s="26" t="s">
         <v>225</v>
       </c>
-      <c r="D113" s="21" t="s">
+      <c r="D113" s="19" t="s">
         <v>337</v>
       </c>
     </row>
     <row r="114" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A114" s="33" t="s">
+      <c r="A114" s="29" t="s">
         <v>338</v>
       </c>
       <c r="B114" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>yusup</v>
-      </c>
-      <c r="C114" s="30" t="s">
-        <v>67</v>
-      </c>
-      <c r="D114" s="21" t="s">
+        <v>adam.akbar</v>
+      </c>
+      <c r="C114" s="27" t="s">
+        <v>349</v>
+      </c>
+      <c r="D114" s="19" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A115" s="29" t="s">
+        <v>339</v>
+      </c>
+      <c r="B115" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>halimatussakdiah</v>
+      </c>
+      <c r="C115" s="27" t="s">
+        <v>350</v>
+      </c>
+      <c r="D115" s="19" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A116" s="29" t="s">
+        <v>340</v>
+      </c>
+      <c r="B116" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>ari.pidada</v>
+      </c>
+      <c r="C116" s="27" t="s">
+        <v>351</v>
+      </c>
+      <c r="D116" s="19" t="s">
         <v>371</v>
       </c>
     </row>
-    <row r="115" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A115" s="34" t="s">
-        <v>339</v>
-      </c>
-      <c r="B115" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>adam.akbar</v>
-      </c>
-      <c r="C115" s="30" t="s">
-        <v>350</v>
-      </c>
-      <c r="D115" s="21" t="s">
+    <row r="117" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A117" s="29" t="s">
+        <v>341</v>
+      </c>
+      <c r="B117" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>alvin.airlangga</v>
+      </c>
+      <c r="C117" s="27" t="s">
+        <v>352</v>
+      </c>
+      <c r="D117" s="19" t="s">
         <v>372</v>
       </c>
     </row>
-    <row r="116" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A116" s="34" t="s">
-        <v>340</v>
-      </c>
-      <c r="B116" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>halimatussakdiah</v>
-      </c>
-      <c r="C116" s="30" t="s">
-        <v>351</v>
-      </c>
-      <c r="D116" s="21" t="s">
+    <row r="118" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A118" s="29" t="s">
+        <v>342</v>
+      </c>
+      <c r="B118" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>savira.putri</v>
+      </c>
+      <c r="C118" s="27" t="s">
+        <v>353</v>
+      </c>
+      <c r="D118" s="19" t="s">
         <v>373</v>
       </c>
     </row>
-    <row r="117" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A117" s="34" t="s">
-        <v>341</v>
-      </c>
-      <c r="B117" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>ari.pidada</v>
-      </c>
-      <c r="C117" s="30" t="s">
-        <v>352</v>
-      </c>
-      <c r="D117" s="21" t="s">
+    <row r="119" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A119" s="29" t="s">
+        <v>343</v>
+      </c>
+      <c r="B119" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>wisnu.dio</v>
+      </c>
+      <c r="C119" s="27" t="s">
+        <v>354</v>
+      </c>
+      <c r="D119" s="19" t="s">
         <v>374</v>
       </c>
     </row>
-    <row r="118" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A118" s="34" t="s">
-        <v>342</v>
-      </c>
-      <c r="B118" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>alvin.airlangga</v>
-      </c>
-      <c r="C118" s="30" t="s">
-        <v>353</v>
-      </c>
-      <c r="D118" s="21" t="s">
+    <row r="120" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A120" s="29" t="s">
+        <v>344</v>
+      </c>
+      <c r="B120" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>aprian.mahendra</v>
+      </c>
+      <c r="C120" s="27" t="s">
+        <v>355</v>
+      </c>
+      <c r="D120" s="19" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="119" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A119" s="34" t="s">
-        <v>343</v>
-      </c>
-      <c r="B119" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>savira.putri</v>
-      </c>
-      <c r="C119" s="30" t="s">
-        <v>354</v>
-      </c>
-      <c r="D119" s="21" t="s">
+    <row r="121" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A121" s="29" t="s">
+        <v>345</v>
+      </c>
+      <c r="B121" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>martha.saptiany</v>
+      </c>
+      <c r="C121" s="27" t="s">
+        <v>356</v>
+      </c>
+      <c r="D121" s="19" t="s">
         <v>376</v>
       </c>
     </row>
-    <row r="120" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A120" s="34" t="s">
-        <v>344</v>
-      </c>
-      <c r="B120" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>wisnu.dio</v>
-      </c>
-      <c r="C120" s="30" t="s">
-        <v>355</v>
-      </c>
-      <c r="D120" s="21" t="s">
+    <row r="122" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A122" s="29" t="s">
+        <v>346</v>
+      </c>
+      <c r="B122" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>wahyu.hadi</v>
+      </c>
+      <c r="C122" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="D122" s="19" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="121" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A121" s="34" t="s">
-        <v>345</v>
-      </c>
-      <c r="B121" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>aprian.mahendra</v>
-      </c>
-      <c r="C121" s="30" t="s">
-        <v>356</v>
-      </c>
-      <c r="D121" s="21" t="s">
+    <row r="123" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A123" s="15" t="s">
+        <v>347</v>
+      </c>
+      <c r="B123" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>zulham.julistiono</v>
+      </c>
+      <c r="C123" s="27" t="s">
+        <v>358</v>
+      </c>
+      <c r="D123" s="19" t="s">
         <v>378</v>
       </c>
     </row>
-    <row r="122" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A122" s="34" t="s">
-        <v>346</v>
-      </c>
-      <c r="B122" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>martha.saptiany</v>
-      </c>
-      <c r="C122" s="30" t="s">
-        <v>357</v>
-      </c>
-      <c r="D122" s="21" t="s">
+    <row r="124" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A124" s="15" t="s">
+        <v>348</v>
+      </c>
+      <c r="B124" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>sulastri.dewi</v>
+      </c>
+      <c r="C124" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="D124" s="19" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="123" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A123" s="34" t="s">
-        <v>347</v>
-      </c>
-      <c r="B123" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>wahyu.hadi</v>
-      </c>
-      <c r="C123" s="30" t="s">
-        <v>358</v>
-      </c>
-      <c r="D123" s="21" t="s">
+    <row r="125" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A125" s="30" t="s">
+        <v>360</v>
+      </c>
+      <c r="B125" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>riki</v>
+      </c>
+      <c r="C125" s="26" t="s">
+        <v>365</v>
+      </c>
+      <c r="D125" s="19" t="s">
         <v>380</v>
       </c>
     </row>
-    <row r="124" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A124" s="16" t="s">
-        <v>348</v>
-      </c>
-      <c r="B124" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>zulham.julistiono</v>
-      </c>
-      <c r="C124" s="30" t="s">
-        <v>359</v>
-      </c>
-      <c r="D124" s="21" t="s">
+    <row r="126" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A126" s="30" t="s">
+        <v>361</v>
+      </c>
+      <c r="B126" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>haris</v>
+      </c>
+      <c r="C126" s="26" t="s">
+        <v>366</v>
+      </c>
+      <c r="D126" s="19" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="125" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A125" s="16" t="s">
-        <v>349</v>
-      </c>
-      <c r="B125" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>sulastri.dewi</v>
-      </c>
-      <c r="C125" s="6" t="s">
-        <v>360</v>
-      </c>
-      <c r="D125" s="21" t="s">
+    <row r="127" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A127" s="9" t="s">
+        <v>362</v>
+      </c>
+      <c r="B127" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>Ertonpati</v>
+      </c>
+      <c r="C127" s="26" t="s">
+        <v>405</v>
+      </c>
+      <c r="D127" s="19" t="s">
         <v>382</v>
-      </c>
-    </row>
-    <row r="126" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A126" s="35" t="s">
-        <v>361</v>
-      </c>
-      <c r="B126" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>riki</v>
-      </c>
-      <c r="C126" s="29" t="s">
-        <v>366</v>
-      </c>
-      <c r="D126" s="21" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="127" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A127" s="35" t="s">
-        <v>362</v>
-      </c>
-      <c r="B127" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>haris</v>
-      </c>
-      <c r="C127" s="29" t="s">
-        <v>367</v>
-      </c>
-      <c r="D127" s="21" t="s">
-        <v>384</v>
       </c>
     </row>
     <row r="128" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
@@ -3833,133 +3822,118 @@
       </c>
       <c r="B128" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>pati</v>
-      </c>
-      <c r="C128" s="29" t="s">
+        <v>yulia</v>
+      </c>
+      <c r="C128" s="26" t="s">
+        <v>367</v>
+      </c>
+      <c r="D128" s="19" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A129" s="31" t="s">
+        <v>364</v>
+      </c>
+      <c r="B129" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>tsabiatun</v>
+      </c>
+      <c r="C129" s="26" t="s">
         <v>368</v>
       </c>
-      <c r="D128" s="21" t="s">
+      <c r="D129" s="19" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A130" s="32" t="s">
         <v>385</v>
       </c>
-    </row>
-    <row r="129" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A129" s="9" t="s">
-        <v>364</v>
-      </c>
-      <c r="B129" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>yulia</v>
-      </c>
-      <c r="C129" s="29" t="s">
-        <v>369</v>
-      </c>
-      <c r="D129" s="21" t="s">
+      <c r="B130" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>imamhadi</v>
+      </c>
+      <c r="C130" s="26" t="s">
+        <v>391</v>
+      </c>
+      <c r="D130" s="19" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A131" s="32" t="s">
         <v>386</v>
       </c>
-    </row>
-    <row r="130" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A130" s="36" t="s">
-        <v>365</v>
-      </c>
-      <c r="B130" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>tsabiatun</v>
-      </c>
-      <c r="C130" s="29" t="s">
-        <v>370</v>
-      </c>
-      <c r="D130" s="21" t="s">
+      <c r="B131" s="2" t="str">
+        <f t="shared" ref="B131:B135" si="2">LEFT(C131, FIND("@", C131) - 1)</f>
+        <v>sitirahayu</v>
+      </c>
+      <c r="C131" s="26" t="s">
+        <v>392</v>
+      </c>
+      <c r="D131" s="19" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A132" s="32" t="s">
         <v>387</v>
       </c>
-    </row>
-    <row r="131" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A131" s="37" t="s">
+      <c r="B132" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>ardiwijaya</v>
+      </c>
+      <c r="C132" s="26" t="s">
+        <v>393</v>
+      </c>
+      <c r="D132" s="19" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="A133" s="32" t="s">
         <v>388</v>
-      </c>
-      <c r="B131" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>imamhadi</v>
-      </c>
-      <c r="C131" s="29" t="s">
-        <v>394</v>
-      </c>
-      <c r="D131" s="21" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="132" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A132" s="37" t="s">
-        <v>389</v>
-      </c>
-      <c r="B132" s="2" t="str">
-        <f t="shared" ref="B132:B136" si="2">LEFT(C132, FIND("@", C132) - 1)</f>
-        <v>sitirahayu</v>
-      </c>
-      <c r="C132" s="29" t="s">
-        <v>395</v>
-      </c>
-      <c r="D132" s="21" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="133" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A133" s="37" t="s">
-        <v>390</v>
       </c>
       <c r="B133" s="2" t="str">
         <f t="shared" si="2"/>
-        <v>ardiwijaya</v>
-      </c>
-      <c r="C133" s="29" t="s">
-        <v>396</v>
-      </c>
-      <c r="D133" s="21" t="s">
-        <v>402</v>
+        <v>ance</v>
+      </c>
+      <c r="C133" s="26" t="s">
+        <v>394</v>
+      </c>
+      <c r="D133" s="19" t="s">
+        <v>400</v>
       </c>
     </row>
     <row r="134" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A134" s="37" t="s">
-        <v>391</v>
+      <c r="A134" s="32" t="s">
+        <v>389</v>
       </c>
       <c r="B134" s="2" t="str">
         <f t="shared" si="2"/>
-        <v>ance</v>
-      </c>
-      <c r="C134" s="29" t="s">
-        <v>397</v>
-      </c>
-      <c r="D134" s="21" t="s">
-        <v>403</v>
+        <v>ziki</v>
+      </c>
+      <c r="C134" s="26" t="s">
+        <v>395</v>
+      </c>
+      <c r="D134" s="19" t="s">
+        <v>401</v>
       </c>
     </row>
     <row r="135" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A135" s="37" t="s">
-        <v>392</v>
+      <c r="A135" s="32" t="s">
+        <v>390</v>
       </c>
       <c r="B135" s="2" t="str">
         <f t="shared" si="2"/>
-        <v>ziki</v>
-      </c>
-      <c r="C135" s="29" t="s">
-        <v>398</v>
-      </c>
-      <c r="D135" s="21" t="s">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="136" spans="1:4" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A136" s="37" t="s">
-        <v>393</v>
-      </c>
-      <c r="B136" s="2" t="str">
-        <f t="shared" si="2"/>
         <v>joni</v>
       </c>
-      <c r="C136" s="29" t="s">
-        <v>399</v>
-      </c>
-      <c r="D136" s="21" t="s">
-        <v>405</v>
+      <c r="C135" s="26" t="s">
+        <v>396</v>
+      </c>
+      <c r="D135" s="19" t="s">
+        <v>402</v>
       </c>
     </row>
   </sheetData>
@@ -4063,31 +4037,30 @@
     <hyperlink ref="C111" r:id="rId96" xr:uid="{8D000EDE-0993-4FB3-9D2F-B6C86DF53679}"/>
     <hyperlink ref="C112" r:id="rId97" xr:uid="{FF0C56D7-58F3-4646-98D4-558B197298DE}"/>
     <hyperlink ref="C113" r:id="rId98" xr:uid="{7EE94315-A543-492D-922B-E3535081B2D5}"/>
-    <hyperlink ref="C114" r:id="rId99" xr:uid="{1947F25C-AAAD-40BC-B3BD-77394A8D7B99}"/>
-    <hyperlink ref="C115" r:id="rId100" xr:uid="{6B115329-92B2-47E1-A3EB-534D4E3F4DC3}"/>
-    <hyperlink ref="C116" r:id="rId101" xr:uid="{DE8B753E-6E9C-4D42-8087-95B0AC7E3FB5}"/>
-    <hyperlink ref="C117" r:id="rId102" xr:uid="{25B91766-0D50-441B-B3B3-41B9075CED13}"/>
-    <hyperlink ref="C118" r:id="rId103" xr:uid="{65888F0C-7CC4-4C1A-8280-0A15695364CA}"/>
-    <hyperlink ref="C119" r:id="rId104" xr:uid="{92BE8DEA-3B34-4CF4-B0EA-8B76CD27E09B}"/>
-    <hyperlink ref="C120" r:id="rId105" xr:uid="{A4D278A8-08D2-4CCB-BBE4-3CBCEC53946E}"/>
-    <hyperlink ref="C121" r:id="rId106" xr:uid="{5866269F-B2DC-410D-A8E2-E27E1A2BDBC1}"/>
-    <hyperlink ref="C122" r:id="rId107" xr:uid="{DF1D79A8-D773-4CAD-81DD-99FFEE90E1BC}"/>
-    <hyperlink ref="C123" r:id="rId108" xr:uid="{9E8E8B2B-AD21-4C0E-91AF-29A337D80CE8}"/>
-    <hyperlink ref="C124" r:id="rId109" xr:uid="{AB53BAF1-D63D-4F53-BBAB-4517B3EAEF8C}"/>
-    <hyperlink ref="C125" r:id="rId110" xr:uid="{5B82A068-FCBF-4B85-922F-357DBAAE5C52}"/>
-    <hyperlink ref="C126" r:id="rId111" xr:uid="{D4999C6E-1807-4E0B-928C-C2296D7D7D67}"/>
-    <hyperlink ref="C127" r:id="rId112" xr:uid="{37D067E3-8C5B-4A6A-AA08-D4A006299185}"/>
-    <hyperlink ref="C128" r:id="rId113" xr:uid="{C871583F-937B-4D54-8D5D-E979FBD29594}"/>
-    <hyperlink ref="C129" r:id="rId114" xr:uid="{E7BF21CA-D632-4AF7-9445-0D66A6F8255F}"/>
-    <hyperlink ref="C130" r:id="rId115" xr:uid="{89EC2F25-7252-49F2-BBE2-D2F378AE4B8C}"/>
-    <hyperlink ref="C131" r:id="rId116" xr:uid="{D8152122-C874-4FFE-8CAC-E4C5B2035BBB}"/>
-    <hyperlink ref="C132" r:id="rId117" xr:uid="{6562668F-4C6B-4ECE-94B0-CB127C94243F}"/>
-    <hyperlink ref="C133" r:id="rId118" xr:uid="{EBE0D7D4-2129-4DFD-9CA9-A8D46173F3AF}"/>
-    <hyperlink ref="C134" r:id="rId119" xr:uid="{53F42B6E-BDD5-4BA7-8D15-F70ACE179A2B}"/>
-    <hyperlink ref="C135" r:id="rId120" xr:uid="{3F6D87B8-7FFF-4254-B2A5-D7A2E194F93A}"/>
-    <hyperlink ref="C136" r:id="rId121" xr:uid="{A33EAB57-7244-4AD1-A54D-C052517179D1}"/>
+    <hyperlink ref="C114" r:id="rId99" xr:uid="{6B115329-92B2-47E1-A3EB-534D4E3F4DC3}"/>
+    <hyperlink ref="C115" r:id="rId100" xr:uid="{DE8B753E-6E9C-4D42-8087-95B0AC7E3FB5}"/>
+    <hyperlink ref="C116" r:id="rId101" xr:uid="{25B91766-0D50-441B-B3B3-41B9075CED13}"/>
+    <hyperlink ref="C117" r:id="rId102" xr:uid="{65888F0C-7CC4-4C1A-8280-0A15695364CA}"/>
+    <hyperlink ref="C118" r:id="rId103" xr:uid="{92BE8DEA-3B34-4CF4-B0EA-8B76CD27E09B}"/>
+    <hyperlink ref="C119" r:id="rId104" xr:uid="{A4D278A8-08D2-4CCB-BBE4-3CBCEC53946E}"/>
+    <hyperlink ref="C120" r:id="rId105" xr:uid="{5866269F-B2DC-410D-A8E2-E27E1A2BDBC1}"/>
+    <hyperlink ref="C121" r:id="rId106" xr:uid="{DF1D79A8-D773-4CAD-81DD-99FFEE90E1BC}"/>
+    <hyperlink ref="C122" r:id="rId107" xr:uid="{9E8E8B2B-AD21-4C0E-91AF-29A337D80CE8}"/>
+    <hyperlink ref="C123" r:id="rId108" xr:uid="{AB53BAF1-D63D-4F53-BBAB-4517B3EAEF8C}"/>
+    <hyperlink ref="C124" r:id="rId109" xr:uid="{5B82A068-FCBF-4B85-922F-357DBAAE5C52}"/>
+    <hyperlink ref="C125" r:id="rId110" xr:uid="{D4999C6E-1807-4E0B-928C-C2296D7D7D67}"/>
+    <hyperlink ref="C126" r:id="rId111" xr:uid="{37D067E3-8C5B-4A6A-AA08-D4A006299185}"/>
+    <hyperlink ref="C127" r:id="rId112" xr:uid="{C871583F-937B-4D54-8D5D-E979FBD29594}"/>
+    <hyperlink ref="C128" r:id="rId113" xr:uid="{E7BF21CA-D632-4AF7-9445-0D66A6F8255F}"/>
+    <hyperlink ref="C129" r:id="rId114" xr:uid="{89EC2F25-7252-49F2-BBE2-D2F378AE4B8C}"/>
+    <hyperlink ref="C130" r:id="rId115" xr:uid="{D8152122-C874-4FFE-8CAC-E4C5B2035BBB}"/>
+    <hyperlink ref="C131" r:id="rId116" xr:uid="{6562668F-4C6B-4ECE-94B0-CB127C94243F}"/>
+    <hyperlink ref="C132" r:id="rId117" xr:uid="{EBE0D7D4-2129-4DFD-9CA9-A8D46173F3AF}"/>
+    <hyperlink ref="C133" r:id="rId118" xr:uid="{53F42B6E-BDD5-4BA7-8D15-F70ACE179A2B}"/>
+    <hyperlink ref="C134" r:id="rId119" xr:uid="{3F6D87B8-7FFF-4254-B2A5-D7A2E194F93A}"/>
+    <hyperlink ref="C135" r:id="rId120" xr:uid="{A33EAB57-7244-4AD1-A54D-C052517179D1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId122"/>
+  <legacyDrawing r:id="rId121"/>
 </worksheet>
 </file>
</xml_diff>